<commit_message>
docs: record R20 pull request and finalize production tracker
</commit_message>
<xml_diff>
--- a/docs/planning/BOW_INTERFACE_SPRITES_R20.xlsx
+++ b/docs/planning/BOW_INTERFACE_SPRITES_R20.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="1" r:id="Rf198707d66f547c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="2" r:id="R9c3d27b772b94990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="3" r:id="R3fdba88c8c164116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="1" r:id="R71ed7c8fe5414ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="2" r:id="Rc3ea55ff75044499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="3" r:id="R68d26e1379904e96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -559,7 +559,7 @@
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="21" t="n">
         <x:f>COUNTIFS(B8:B1000,"Livraison R20",D8:D1000,"VALIDÉ")</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="21" t="n">
@@ -884,17 +884,17 @@
         <x:v>Publication de la continuation</x:v>
       </x:c>
       <x:c r="D19" s="18" t="str">
-        <x:v>EN COURS</x:v>
+        <x:v>VALIDÉ</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>Branche R20 fondée sur R18 fusionnée et R19 conservée.</x:v>
+        <x:v>Branche codex/r20-player-shell-sprites publiée avec code, rapports et Excel; PR #14 ouverte.</x:v>
       </x:c>
       <x:c r="F19" s="18" t="str">
-        <x:v>Publier le commit vérifié et la PR de continuation.</x:v>
+        <x:v>Revue humaine et suite de production ; résultats CI consultables sur la PR.</x:v>
       </x:c>
       <x:c r="G19" s="18" t="str">
-        <x:v>codex/r20-player-shell-sprites
-Source : GitHub darknigthmare/resident-evil-bow-protocol</x:v>
+        <x:v>https://github.com/darknigthmare/resident-evil-bow-protocol/pull/14
+Source : Commit initial 928d07b9; arbre identique au candidat testé</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="56" customHeight="1">
@@ -1247,10 +1247,10 @@
         <x:v>EN COURS</x:v>
       </x:c>
       <x:c r="E34" s="17" t="str">
-        <x:v>R8 à R19 conservées et nouveau suivi lié au code.</x:v>
+        <x:v>R8 à R19 conservées; R20 publiée avec code, rapports et classeur dans la PR #14.</x:v>
       </x:c>
       <x:c r="F34" s="17" t="str">
-        <x:v>Publication R20, CI finale et livraisons futures, sans déclarer le jeu complet.</x:v>
+        <x:v>Revue humaine et livraisons futures ; résultats CI consultables sur la PR. Les lots globaux restent ouverts.</x:v>
       </x:c>
       <x:c r="G34" s="17" t="str">
         <x:v>docs/R20_TRACKING.json
@@ -1282,7 +1282,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8c2399e76f44f6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdc62fffa07f4431"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14673,7 +14673,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc213ae07fd4f4ba0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ffe24fb6b5947e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15250,7 +15250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34dedba9016c48ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6390fe8df9c445ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>